<commit_message>
update table1-15 with 合計 column
</commit_message>
<xml_diff>
--- a/table1-15.xlsx
+++ b/table1-15.xlsx
@@ -488,7 +488,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>表1-15、115年各身分別對個別資料庫感到滿意的比例排行（依表1-13滿意比例 / 整體使用率依表1-5，均從原始問卷RAW重算）</t>
+          <t>表1-15、115年各身分別對個別資料庫感到滿意的比例排行（依表1-13滿意比例，從原始問卷RAW重算；第四欄為表1-13合計）</t>
         </is>
       </c>
     </row>
@@ -510,7 +510,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>整體使用率排行</t>
+          <t>合計滿意度排行(全身份)</t>
         </is>
       </c>
     </row>
@@ -615,11 +615,11 @@
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>空中英語教室影音典藏學習系統-空中英語教室每日頻道</t>
+          <t>LiveABC英日語AI互動學習資料庫</t>
         </is>
       </c>
       <c r="L4" s="4" t="n">
-        <v>67.06</v>
+        <v>84.05</v>
       </c>
     </row>
     <row r="5">
@@ -661,11 +661,11 @@
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>LiveABC英日語AI互動學習資料庫</t>
+          <t>空中英語教室影音典藏學習系統-空中英語教室每日頻道</t>
         </is>
       </c>
       <c r="L5" s="4" t="n">
-        <v>66.15000000000001</v>
+        <v>83.45</v>
       </c>
     </row>
     <row r="6">
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>65.5</v>
+        <v>83.33</v>
       </c>
     </row>
     <row r="7">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>64.22</v>
+        <v>82.43000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -799,11 +799,11 @@
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>哈佛商業評論影音知識庫</t>
+          <t>AEB 電子雜誌出版服務平台-Walking Library 電子雜誌</t>
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>63.21</v>
+        <v>80.41</v>
       </c>
     </row>
     <row r="9">
@@ -845,11 +845,11 @@
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>AEB 電子雜誌出版服務平台-Walking Library 電子雜誌</t>
+          <t>Web of Science AI智能核心合輯資料庫</t>
         </is>
       </c>
       <c r="L9" s="4" t="n">
-        <v>63.21</v>
+        <v>79.88</v>
       </c>
     </row>
     <row r="10">
@@ -895,7 +895,7 @@
         </is>
       </c>
       <c r="L10" s="4" t="n">
-        <v>62.84</v>
+        <v>79.27</v>
       </c>
     </row>
     <row r="11">
@@ -937,11 +937,11 @@
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>Web of Science AI智能核心合輯資料庫</t>
+          <t>外文雜誌精選平台</t>
         </is>
       </c>
       <c r="L11" s="4" t="n">
-        <v>61.56</v>
+        <v>78.62</v>
       </c>
     </row>
     <row r="12">
@@ -983,11 +983,11 @@
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>InCites™ Journal Citation Reports (JCR)</t>
+          <t>哈佛商業評論影音知識庫</t>
         </is>
       </c>
       <c r="L12" s="4" t="n">
-        <v>61.47</v>
+        <v>78.52</v>
       </c>
     </row>
     <row r="13">
@@ -1029,11 +1029,11 @@
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>外文雜誌精選平台</t>
+          <t>InCites™ Journal Citation Reports (JCR)</t>
         </is>
       </c>
       <c r="L13" s="4" t="n">
-        <v>61.38</v>
+        <v>77.76000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -1079,13 +1079,13 @@
         </is>
       </c>
       <c r="L14" s="4" t="n">
-        <v>59.63</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>註：前三欄為各身分「曾使用過人數」為分母之滿意比例（滿意+非常滿意）；第四欄為各資料庫「曾使用人數÷總填答1090」之整體使用率。以上均直接從原始問卷 20260601 重算，非衍生檔。</t>
+          <t>註：前3欄為各身分「曾使用過人數」為分母之滿意比例（滿意+非常滿意）；第四欄「合計」為全身份（含職員、研究人員）之整體滿意比例，分母=曾使用過該庫之人數。均直接從原始問卷20260601 RAW重算。</t>
         </is>
       </c>
     </row>

</xml_diff>